<commit_message>
feat(samples): add an Instructions sheet to the template
Explains each column with an example and how to bring data from separate opening, closing and sales files with BUSCARX. The data sheet stays first, which is the one Matices reads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mvp-matices/data/sample/plantilla-matices.xlsx
+++ b/mvp-matices/data/sample/plantilla-matices.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Inventario"/>
+    <sheet r:id="rId2" sheetId="2" name="Instrucciones"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -59,6 +60,105 @@
   </si>
   <si>
     <t>TINTE CREMA AURA 1 NEGRO 60 ML</t>
+  </si>
+  <si>
+    <t>Plantilla Matices: cómo llenarla</t>
+  </si>
+  <si>
+    <t>1. Llena la hoja Inventario: una fila por producto y por periodo. No cambies los nombres de las columnas.</t>
+  </si>
+  <si>
+    <t>2. Para varios periodos (por ejemplo julio, agosto y septiembre) agrega más filas con sus fechas, en la misma hoja.</t>
+  </si>
+  <si>
+    <t>3. Guarda como .xlsx (recomendado) o .csv y cárgalo en Matices. Deja la hoja Inventario como primera hoja.</t>
+  </si>
+  <si>
+    <t>Columna</t>
+  </si>
+  <si>
+    <t>Obligatoria</t>
+  </si>
+  <si>
+    <t>Qué poner</t>
+  </si>
+  <si>
+    <t>Ejemplo</t>
+  </si>
+  <si>
+    <t>Sí</t>
+  </si>
+  <si>
+    <t>Primer día del periodo, AAAA-MM-DD o DD/MM/AAAA</t>
+  </si>
+  <si>
+    <t>Último día del periodo</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Código del producto en tu sistema. Si no lo tienes, déjalo vacío: el producto se identifica por su nombre</t>
+  </si>
+  <si>
+    <t>Nombre del producto, escrito igual en todos los periodos</t>
+  </si>
+  <si>
+    <t>Unidades al inicio del periodo (número entero)</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Unidades al final del periodo (número entero)</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Unidades vendidas entre periodo_inicio y periodo_fin</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Unidades el día del análisis. Si no tienes la columna, bórrala: se usa el inventario final</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Unidades pedidas que aún no llegan. Vacío = 0</t>
+  </si>
+  <si>
+    <t>Costo por unidad en pesos, sin puntos de miles ni $</t>
+  </si>
+  <si>
+    <t>9200</t>
+  </si>
+  <si>
+    <t>Precio de venta por unidad en pesos</t>
+  </si>
+  <si>
+    <t>16900</t>
+  </si>
+  <si>
+    <t>Si tus datos vienen en archivos separados (inventario inicial, inventario final y ventas):</t>
+  </si>
+  <si>
+    <t>a. Copia la lista de productos en la columna producto.</t>
+  </si>
+  <si>
+    <t>b. Trae cada cantidad buscando por nombre, por ejemplo en inventario_final:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   =BUSCARX(D2;'[INV FINAL AGO.xlsx]Hoja1'!$A:$A;'[INV FINAL AGO.xlsx]Hoja1'!$B:$B;"NO ESTÁ")</t>
+  </si>
+  <si>
+    <t>c. Revisa que ningún producto diga NO ESTÁ y pega las columnas como valores antes de guardar.</t>
+  </si>
+  <si>
+    <t>Matices recomienda; no compra. Cada compra la decide y aprueba una persona.</t>
   </si>
 </sst>
 </file>
@@ -170,4 +270,239 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="90" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>